<commit_message>
added simple car schematic
</commit_message>
<xml_diff>
--- a/14.10_NXP_Kit_List.xlsx
+++ b/14.10_NXP_Kit_List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Desktop\FH Joanneum\Sem5\Projektarbeit\Programming\NXPCar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6C14252-B934-4C46-AF86-B27D24B002FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A6550F-CB8D-4411-AFC8-D5BCBF9D1226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D6B5232E-38FB-4653-99FB-33D748289929}"/>
+    <workbookView xWindow="-14505" yWindow="-1050" windowWidth="14610" windowHeight="15585" xr2:uid="{D6B5232E-38FB-4653-99FB-33D748289929}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>Name</t>
   </si>
@@ -227,13 +227,10 @@
     <t>425-2062-ND</t>
   </si>
   <si>
-    <t>TCRT5000</t>
-  </si>
-  <si>
-    <t>751-1033-5-ND</t>
-  </si>
-  <si>
     <t>Optischer Sensor</t>
+  </si>
+  <si>
+    <t>1528-2395-ND</t>
   </si>
 </sst>
 </file>
@@ -671,7 +668,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -725,10 +722,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="2" t="s">
         <v>62</v>
+      </c>
+      <c r="C6" s="2">
+        <v>3595</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>63</v>

</xml_diff>